<commit_message>
maj site complet 25/07/2026
</commit_message>
<xml_diff>
--- a/Produit/Produit.xlsx
+++ b/Produit/Produit.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Theina3D\Theina3D\Produit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{490FA8C6-FFE6-4BB1-8689-AD70771CB219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7CC5117-D1FC-45F0-A7E1-97EAB6A99005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C8E30C7B-B677-4B82-9030-6930B4140F13}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{C8E30C7B-B677-4B82-9030-6930B4140F13}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet name="Calculs &amp; Barème" sheetId="2" r:id="rId2"/>
+    <sheet name="Devis Client" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="107">
   <si>
     <t>Skadis_Casque_Support - Part 1</t>
   </si>
@@ -141,16 +143,246 @@
   </si>
   <si>
     <t>% dons</t>
+  </si>
+  <si>
+    <t>1kg &lt; Colis &lt; 3kg</t>
+  </si>
+  <si>
+    <t>Colis &lt; 1kg</t>
+  </si>
+  <si>
+    <t>Marge Livraison (€)</t>
+  </si>
+  <si>
+    <t>Facturé au Client (€)</t>
+  </si>
+  <si>
+    <t>Payé au Fournisseur (€)</t>
+  </si>
+  <si>
+    <t>Type Colis / Tranche</t>
+  </si>
+  <si>
+    <t>4. Grille Expédition &amp; Livraison Proto</t>
+  </si>
+  <si>
+    <t>TOTAL Impression Prototype</t>
+  </si>
+  <si>
+    <t>Coût Usure &amp; Maintenance Machine</t>
+  </si>
+  <si>
+    <t>Coût Électricité</t>
+  </si>
+  <si>
+    <t>Coût Matière (Filament)</t>
+  </si>
+  <si>
+    <t>hh:mm:ss</t>
+  </si>
+  <si>
+    <t>06:31:00</t>
+  </si>
+  <si>
+    <t>Temps d'impression</t>
+  </si>
+  <si>
+    <t>grammes (g)</t>
+  </si>
+  <si>
+    <t>Poids de filament utilisé</t>
+  </si>
+  <si>
+    <t>Marge Nette</t>
+  </si>
+  <si>
+    <t>Cotisations URSSAF</t>
+  </si>
+  <si>
+    <t>Prix de Vente Estimé</t>
+  </si>
+  <si>
+    <t>Calcul Coût de Revient</t>
+  </si>
+  <si>
+    <t>Unité / Formule</t>
+  </si>
+  <si>
+    <t>Valeur</t>
+  </si>
+  <si>
+    <t>Paramètre Impression</t>
+  </si>
+  <si>
+    <t>3. Calculateur Impression Prototype 3D</t>
+  </si>
+  <si>
+    <t>Livraison des fichiers (STEP, STL, DWG)</t>
+  </si>
+  <si>
+    <t>Conception technique</t>
+  </si>
+  <si>
+    <t>Reproduction technique</t>
+  </si>
+  <si>
+    <t>Conception simple</t>
+  </si>
+  <si>
+    <t>Prix de Vente (PV)</t>
+  </si>
+  <si>
+    <t>Coût de Revient</t>
+  </si>
+  <si>
+    <t>Temps (h)</t>
+  </si>
+  <si>
+    <t>Taux Horaire (€/h)</t>
+  </si>
+  <si>
+    <t>Prestation</t>
+  </si>
+  <si>
+    <t>2. Grille Tarifaire Conception CAO / 3D</t>
+  </si>
+  <si>
+    <t>Prix moyen bobine 1kg</t>
+  </si>
+  <si>
+    <t>Prix filament PLA / kg</t>
+  </si>
+  <si>
+    <t>Puissance moyenne en Watts (W)</t>
+  </si>
+  <si>
+    <t>Consommation moyenne imprimante</t>
+  </si>
+  <si>
+    <t>Tarif moyen TTC du kWh</t>
+  </si>
+  <si>
+    <t>Prix du kWh d'électricité</t>
+  </si>
+  <si>
+    <t>Maintenance + amortissement machine</t>
+  </si>
+  <si>
+    <t>Coût usure machine / heure</t>
+  </si>
+  <si>
+    <t>Taux URSSAF / Micro-entreprise</t>
+  </si>
+  <si>
+    <t>Taux de cotisation sociale</t>
+  </si>
+  <si>
+    <t>Unité / Note</t>
+  </si>
+  <si>
+    <t>Désignation</t>
+  </si>
+  <si>
+    <t>1. Taux de Cotisation, Électricité &amp; Usure Machine</t>
+  </si>
+  <si>
+    <t>PARAMÈTRES DE CALCUL, COÛTS DE REVIENT &amp; MARGES</t>
+  </si>
+  <si>
+    <t>NOTE IMPORTANTE CONCERNANT LE PROTOTYPE 3D :
+Le chiffrage du prototype imprimé (option PRT-3D) est une estimation prévisionnelle basée sur l'analyse initiale de votre besoin.
+Le fichier 3D définitif n'étant pas encore généré au moment de ce devis, le montant du prototype est délibérément estimé avec une marge de sécurité. Lors de la livraison finale du fichier et du lancement de l'impression, le tarif pourra être RÉAJUSTÉ À LA BAISSE si le coût de revient réel (temps d'impression effectif, consommation électrique et poids de matière) s'avère inférieur aux prévisions.</t>
+  </si>
+  <si>
+    <t>Net à payer (€) :</t>
+  </si>
+  <si>
+    <t>TVA (Franchise) :</t>
+  </si>
+  <si>
+    <t>Total HT :</t>
+  </si>
+  <si>
+    <t>Oui</t>
+  </si>
+  <si>
+    <t>Frais de port &amp; emballage sécurisé (Colis &lt; 1kg)</t>
+  </si>
+  <si>
+    <t>SHP-01</t>
+  </si>
+  <si>
+    <t>Impression 3D - Prototype physique (Cotation estimée)</t>
+  </si>
+  <si>
+    <t>PRT-3D</t>
+  </si>
+  <si>
+    <t>Livraison des fichiers sources &amp; fabrication (STEP, STL, DWG)</t>
+  </si>
+  <si>
+    <t>CAD-DEL</t>
+  </si>
+  <si>
+    <t>Prestation de conception / modélisation 3D</t>
+  </si>
+  <si>
+    <t>CAD-01</t>
+  </si>
+  <si>
+    <t>Total HT</t>
+  </si>
+  <si>
+    <t>Prix Unitaire HT</t>
+  </si>
+  <si>
+    <t>Qté</t>
+  </si>
+  <si>
+    <t>Inclus / Option</t>
+  </si>
+  <si>
+    <t>Description de la prestation</t>
+  </si>
+  <si>
+    <t>Réf / Item</t>
+  </si>
+  <si>
+    <t>SÉLECTION ET DÉTAIL DES PRESTATIONS</t>
+  </si>
+  <si>
+    <t>Nom Client / Société : Client exemple
+Adresse : 45 Avenue des Projets
+Email : client@email.com
+Date du devis : 21/07/2026
+N° Devis : DEV-2026-001</t>
+  </si>
+  <si>
+    <t>Mon Entreprise 3D / Design
+Adresse : 123 Rue de l'Innovation
+Email : contact@monentreprise3d.fr
+N° SIRET : 123 456 789 00012</t>
+  </si>
+  <si>
+    <t>INFORMATIONS CLIENT</t>
+  </si>
+  <si>
+    <t>INFORMATIONS PRESTATAIRE</t>
+  </si>
+  <si>
+    <t>DEVIS DE PRESTATION &amp; PROTOTYPAGE 3D</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00\ \€"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -181,8 +413,43 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0F172A"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF1B365D"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF0F172A"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF475569"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -207,13 +474,61 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
+        <bgColor rgb="FFFEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1B365D"/>
+        <bgColor rgb="FF1B365D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1F5F9"/>
+        <bgColor rgb="FFF1F5F9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1B365D"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -222,28 +537,27 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="3" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -258,6 +572,81 @@
     <xf numFmtId="44" fontId="3" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Monétaire" xfId="1" builtinId="4"/>
@@ -265,81 +654,6 @@
     <cellStyle name="Pourcentage" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="18">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF434343"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF333333"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -378,56 +692,6 @@
         <vertAlign val="baseline"/>
         <sz val="11"/>
         <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="none"/>
@@ -602,6 +866,81 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
+        <color rgb="FF434343"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF333333"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
         <color theme="1"/>
         <name val="Calibri"/>
         <family val="2"/>
@@ -715,6 +1054,56 @@
       </fill>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -729,33 +1118,33 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{96A71FAF-F61C-4F8A-ADB5-40418E571C3E}" name="Tableau1" displayName="Tableau1" ref="A1:P7" totalsRowShown="0" headerRowDxfId="6" dataDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{96A71FAF-F61C-4F8A-ADB5-40418E571C3E}" name="Tableau1" displayName="Tableau1" ref="A1:P7" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
   <autoFilter ref="A1:P7" xr:uid="{96A71FAF-F61C-4F8A-ADB5-40418E571C3E}"/>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{23D466F6-9B2B-4653-93E6-139FE75B4231}" name="SKU" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{595C2037-E6C0-4AAD-95EC-4AA427A537CB}" name="Produit" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{D62D05D7-07D0-4919-88F4-EB47F77F9BB9}" name="bicolor" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{3F1A66C0-8A4C-4B23-845F-EA86C89256ED}" name="Poids" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{2557664B-2D47-4814-A763-E0E1CA9E4242}" name="temps" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{C5622246-3EC6-4575-9B6D-426A7ACD3AB2}" name="cout de revient" dataDxfId="2" dataCellStyle="Monétaire">
+    <tableColumn id="1" xr3:uid="{23D466F6-9B2B-4653-93E6-139FE75B4231}" name="SKU" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{595C2037-E6C0-4AAD-95EC-4AA427A537CB}" name="Produit" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{D62D05D7-07D0-4919-88F4-EB47F77F9BB9}" name="bicolor" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{3F1A66C0-8A4C-4B23-845F-EA86C89256ED}" name="Poids" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{2557664B-2D47-4814-A763-E0E1CA9E4242}" name="temps" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{C5622246-3EC6-4575-9B6D-426A7ACD3AB2}" name="cout de revient" dataDxfId="10" dataCellStyle="Monétaire">
       <calculatedColumnFormula>((D2*($T$1/1000))+(E2*24*(0.15*$T$2))+(E2*24*$T$3))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{3910BEF2-95A1-4E9E-8961-6C9E62FD56D8}" name="PVU" dataDxfId="0" dataCellStyle="Monétaire"/>
-    <tableColumn id="8" xr3:uid="{5667F4D7-744F-4926-889F-132E669CEAEA}" name="Cotisation" dataDxfId="1" dataCellStyle="Monétaire">
+    <tableColumn id="7" xr3:uid="{3910BEF2-95A1-4E9E-8961-6C9E62FD56D8}" name="PVU" dataDxfId="9" dataCellStyle="Monétaire"/>
+    <tableColumn id="8" xr3:uid="{5667F4D7-744F-4926-889F-132E669CEAEA}" name="Cotisation" dataDxfId="8" dataCellStyle="Monétaire">
       <calculatedColumnFormula>Tableau1[[#This Row],[PVU]]*$T$4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{CD65628A-964D-4889-937B-134D75F3696D}" name="bénéfice" dataDxfId="12" dataCellStyle="Monétaire">
+    <tableColumn id="9" xr3:uid="{CD65628A-964D-4889-937B-134D75F3696D}" name="bénéfice" dataDxfId="7" dataCellStyle="Monétaire">
       <calculatedColumnFormula>G2-H2-F2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{909AFF64-52A4-40A9-B0CA-7DD349AA9DFB}" name="image" dataDxfId="11"/>
-    <tableColumn id="11" xr3:uid="{DFF6FB60-F3E2-40F2-BE61-B9B72A71B8BB}" name="poid bicolor 1" dataDxfId="10"/>
-    <tableColumn id="12" xr3:uid="{B22C8D62-1762-47B1-868F-E1CB6C31AD04}" name="poids bicolor 2" dataDxfId="9"/>
-    <tableColumn id="13" xr3:uid="{DBAACC8F-D4F2-4FAF-8CBD-6D390EF0E03D}" name="surcout" dataDxfId="8"/>
-    <tableColumn id="14" xr3:uid="{77ABA3A0-5131-46C3-85CF-053059CD7D4C}" name="dont asso" dataDxfId="5" dataCellStyle="Monétaire">
+    <tableColumn id="10" xr3:uid="{909AFF64-52A4-40A9-B0CA-7DD349AA9DFB}" name="image" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{DFF6FB60-F3E2-40F2-BE61-B9B72A71B8BB}" name="poid bicolor 1" dataDxfId="5"/>
+    <tableColumn id="12" xr3:uid="{B22C8D62-1762-47B1-868F-E1CB6C31AD04}" name="poids bicolor 2" dataDxfId="4"/>
+    <tableColumn id="13" xr3:uid="{DBAACC8F-D4F2-4FAF-8CBD-6D390EF0E03D}" name="surcout" dataDxfId="3"/>
+    <tableColumn id="14" xr3:uid="{77ABA3A0-5131-46C3-85CF-053059CD7D4C}" name="dont asso" dataDxfId="2" dataCellStyle="Monétaire">
       <calculatedColumnFormula>Tableau1[[#This Row],[bénéfice]]*Tableau1[[#This Row],[% dons]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{28BE90EF-3EE9-43DD-B14E-51170F2B8F80}" name="% dons" dataDxfId="4" dataCellStyle="Pourcentage"/>
-    <tableColumn id="15" xr3:uid="{5D676FDF-152E-43F4-8A6D-6A68FD4112A5}" name="bénéfice apres dons" dataDxfId="3" dataCellStyle="Monétaire">
+    <tableColumn id="16" xr3:uid="{28BE90EF-3EE9-43DD-B14E-51170F2B8F80}" name="% dons" dataDxfId="1" dataCellStyle="Pourcentage"/>
+    <tableColumn id="15" xr3:uid="{5D676FDF-152E-43F4-8A6D-6A68FD4112A5}" name="bénéfice apres dons" dataDxfId="0" dataCellStyle="Monétaire">
       <calculatedColumnFormula>Tableau1[[#This Row],[bénéfice]]-Tableau1[[#This Row],[dont asso]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1083,633 +1472,631 @@
   <dimension ref="A1:Y15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="7" width="11.42578125" style="1"/>
-    <col min="8" max="9" width="12.140625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="13.42578125" style="1" customWidth="1"/>
-    <col min="11" max="13" width="12.5703125" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="11.42578125" style="1"/>
+    <col min="8" max="9" width="12.140625" customWidth="1"/>
+    <col min="10" max="10" width="13.42578125" customWidth="1"/>
+    <col min="11" max="13" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="K1" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="L1" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="M1" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="8" t="s">
+      <c r="N1" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="O1" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="P1" s="8" t="s">
+      <c r="P1" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="Q1" s="3"/>
-      <c r="R1" s="3"/>
-      <c r="S1" s="3" t="s">
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="T1" s="4">
+      <c r="T1" s="3">
         <v>25</v>
       </c>
-      <c r="U1" s="3"/>
-      <c r="V1" s="3"/>
-      <c r="W1" s="3"/>
-      <c r="X1" s="3"/>
-      <c r="Y1" s="3"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
+      <c r="X1" s="2"/>
+      <c r="Y1" s="2"/>
     </row>
     <row r="2" spans="1:25" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="1">
         <v>15.75</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>5.7638888888888892E-2</v>
       </c>
-      <c r="F2" s="10">
-        <f>((D2*($T$1/1000))+(E2*24*(0.15*$T$2))+(E2*24*$T$3))</f>
+      <c r="F2" s="9">
+        <f t="shared" ref="F2:F7" si="0">((D2*($T$1/1000))+(E2*24*(0.15*$T$2))+(E2*24*$T$3))</f>
         <v>0.64620833333333338</v>
       </c>
-      <c r="G2" s="12">
+      <c r="G2" s="11">
         <v>5</v>
       </c>
-      <c r="H2" s="10">
+      <c r="H2" s="9">
         <f>Tableau1[[#This Row],[PVU]]*$T$4</f>
         <v>1.06</v>
       </c>
-      <c r="I2" s="10">
+      <c r="I2" s="9">
         <f>G2-H2-F2</f>
         <v>3.2937916666666665</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="10">
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="9">
         <f>Tableau1[[#This Row],[bénéfice]]*Tableau1[[#This Row],[% dons]]</f>
         <v>0.32937916666666667</v>
       </c>
-      <c r="O2" s="9">
+      <c r="O2" s="8">
         <v>0.1</v>
       </c>
-      <c r="P2" s="11">
+      <c r="P2" s="10">
         <f>Tableau1[[#This Row],[bénéfice]]-Tableau1[[#This Row],[dont asso]]</f>
         <v>2.9644124999999999</v>
       </c>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="3"/>
-      <c r="S2" s="3" t="s">
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="T2" s="4">
+      <c r="T2" s="3">
         <v>0.15</v>
       </c>
-      <c r="U2" s="3"/>
-      <c r="V2" s="3"/>
-      <c r="W2" s="3"/>
-      <c r="X2" s="3"/>
-      <c r="Y2" s="3"/>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
+      <c r="W2" s="2"/>
+      <c r="X2" s="2"/>
+      <c r="Y2" s="2"/>
     </row>
     <row r="3" spans="1:25" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="1">
         <v>144.35</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>0.27152777777777776</v>
       </c>
-      <c r="F3" s="10">
-        <f>((D3*($T$1/1000))+(E3*24*(0.15*$T$2))+(E3*24*$T$3))</f>
+      <c r="F3" s="9">
+        <f t="shared" si="0"/>
         <v>4.7980416666666663</v>
       </c>
-      <c r="G3" s="12">
+      <c r="G3" s="11">
         <v>15</v>
       </c>
-      <c r="H3" s="10">
+      <c r="H3" s="9">
         <f>Tableau1[[#This Row],[PVU]]*$T$4</f>
         <v>3.1799999999999997</v>
       </c>
-      <c r="I3" s="10">
+      <c r="I3" s="9">
         <f>G3-H3-F3</f>
         <v>7.021958333333334</v>
       </c>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="10">
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="9">
         <f>Tableau1[[#This Row],[bénéfice]]*Tableau1[[#This Row],[% dons]]</f>
         <v>0.70219583333333346</v>
       </c>
-      <c r="O3" s="9">
+      <c r="O3" s="8">
         <v>0.1</v>
       </c>
-      <c r="P3" s="11">
+      <c r="P3" s="10">
         <f>Tableau1[[#This Row],[bénéfice]]-Tableau1[[#This Row],[dont asso]]</f>
         <v>6.3197625000000004</v>
       </c>
-      <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
-      <c r="S3" s="3" t="s">
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="T3" s="4">
+      <c r="T3" s="3">
         <v>0.16</v>
       </c>
-      <c r="W3" s="3"/>
-      <c r="X3" s="3"/>
-      <c r="Y3" s="3"/>
+      <c r="W3" s="2"/>
+      <c r="X3" s="2"/>
+      <c r="Y3" s="2"/>
     </row>
     <row r="4" spans="1:25" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>1.17</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>0.16250000000000001</v>
       </c>
-      <c r="F4" s="10">
-        <f>((D4*($T$1/1000))+(E4*24*(0.15*$T$2))+(E4*24*$T$3))</f>
+      <c r="F4" s="9">
+        <f t="shared" si="0"/>
         <v>0.7410000000000001</v>
       </c>
-      <c r="G4" s="12">
+      <c r="G4" s="11">
         <v>2</v>
       </c>
-      <c r="H4" s="10">
+      <c r="H4" s="9">
         <f>Tableau1[[#This Row],[PVU]]*$T$4</f>
         <v>0.42399999999999999</v>
       </c>
-      <c r="I4" s="10">
-        <f t="shared" ref="I4:I7" si="0">G4-H4-F4</f>
+      <c r="I4" s="9">
+        <f t="shared" ref="I4:I7" si="1">G4-H4-F4</f>
         <v>0.83499999999999996</v>
       </c>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="10">
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="9">
         <f>Tableau1[[#This Row],[bénéfice]]*Tableau1[[#This Row],[% dons]]</f>
         <v>0.41749999999999998</v>
       </c>
-      <c r="O4" s="9">
+      <c r="O4" s="8">
         <v>0.5</v>
       </c>
-      <c r="P4" s="11">
+      <c r="P4" s="10">
         <f>Tableau1[[#This Row],[bénéfice]]-Tableau1[[#This Row],[dont asso]]</f>
         <v>0.41749999999999998</v>
       </c>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3" t="s">
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="T4" s="3">
+      <c r="T4" s="2">
         <v>0.21199999999999999</v>
       </c>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
-      <c r="Y4" s="3"/>
+      <c r="W4" s="2"/>
+      <c r="X4" s="2"/>
+      <c r="Y4" s="2"/>
     </row>
     <row r="5" spans="1:25" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="1">
         <v>18.440000000000001</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>3.0555555555555555E-2</v>
       </c>
-      <c r="F5" s="10">
-        <f>((D5*($T$1/1000))+(E5*24*(0.15*$T$2))+(E5*24*$T$3))</f>
+      <c r="F5" s="9">
+        <f t="shared" si="0"/>
         <v>0.59483333333333344</v>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="11">
         <v>5</v>
       </c>
-      <c r="H5" s="10">
+      <c r="H5" s="9">
         <f>Tableau1[[#This Row],[PVU]]*$T$4</f>
         <v>1.06</v>
       </c>
-      <c r="I5" s="10">
-        <f t="shared" si="0"/>
+      <c r="I5" s="9">
+        <f t="shared" si="1"/>
         <v>3.3451666666666666</v>
       </c>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2">
+      <c r="J5" s="1"/>
+      <c r="K5" s="1">
         <v>12.74</v>
       </c>
-      <c r="L5" s="2">
+      <c r="L5" s="1">
         <v>5.71</v>
       </c>
-      <c r="M5" s="2">
+      <c r="M5" s="1">
         <v>1</v>
       </c>
-      <c r="N5" s="10">
+      <c r="N5" s="9">
         <f>Tableau1[[#This Row],[bénéfice]]*Tableau1[[#This Row],[% dons]]</f>
         <v>0.33451666666666668</v>
       </c>
-      <c r="O5" s="9">
+      <c r="O5" s="8">
         <v>0.1</v>
       </c>
-      <c r="P5" s="11">
+      <c r="P5" s="10">
         <f>Tableau1[[#This Row],[bénéfice]]-Tableau1[[#This Row],[dont asso]]</f>
         <v>3.01065</v>
       </c>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
-      <c r="T5" s="3"/>
-      <c r="W5" s="3"/>
-      <c r="X5" s="3"/>
-      <c r="Y5" s="3"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="2"/>
+      <c r="T5" s="2"/>
+      <c r="W5" s="2"/>
+      <c r="X5" s="2"/>
+      <c r="Y5" s="2"/>
     </row>
     <row r="6" spans="1:25" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="1">
         <v>18.399999999999999</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>6.5277777777777782E-2</v>
       </c>
-      <c r="F6" s="10">
-        <f>((D6*($T$1/1000))+(E6*24*(0.15*$T$2))+(E6*24*$T$3))</f>
+      <c r="F6" s="9">
+        <f t="shared" si="0"/>
         <v>0.74591666666666667</v>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="11">
         <v>4</v>
       </c>
-      <c r="H6" s="10">
+      <c r="H6" s="9">
         <f>Tableau1[[#This Row],[PVU]]*$T$4</f>
         <v>0.84799999999999998</v>
       </c>
-      <c r="I6" s="10">
-        <f t="shared" si="0"/>
+      <c r="I6" s="9">
+        <f t="shared" si="1"/>
         <v>2.4060833333333336</v>
       </c>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="10">
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="9">
         <f>Tableau1[[#This Row],[bénéfice]]*Tableau1[[#This Row],[% dons]]</f>
         <v>0.24060833333333337</v>
       </c>
-      <c r="O6" s="9">
+      <c r="O6" s="8">
         <v>0.1</v>
       </c>
-      <c r="P6" s="11">
+      <c r="P6" s="10">
         <f>Tableau1[[#This Row],[bénéfice]]-Tableau1[[#This Row],[dont asso]]</f>
         <v>2.1654750000000003</v>
       </c>
-      <c r="Q6" s="3"/>
-      <c r="R6" s="3"/>
-      <c r="S6" s="3"/>
-      <c r="T6" s="3"/>
-      <c r="U6" s="3"/>
-      <c r="V6" s="3"/>
-      <c r="W6" s="3"/>
-      <c r="X6" s="3"/>
-      <c r="Y6" s="3"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="2"/>
+      <c r="W6" s="2"/>
+      <c r="X6" s="2"/>
+      <c r="Y6" s="2"/>
     </row>
     <row r="7" spans="1:25" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="1">
         <v>18.86</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="6">
         <v>7.9861111111111105E-2</v>
       </c>
-      <c r="F7" s="10">
-        <f>((D7*($T$1/1000))+(E7*24*(0.15*$T$2))+(E7*24*$T$3))</f>
+      <c r="F7" s="9">
+        <f t="shared" si="0"/>
         <v>0.82129166666666664</v>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="11">
         <v>4</v>
       </c>
-      <c r="H7" s="10">
+      <c r="H7" s="9">
         <f>Tableau1[[#This Row],[PVU]]*$T$4</f>
         <v>0.84799999999999998</v>
       </c>
-      <c r="I7" s="10">
-        <f t="shared" si="0"/>
+      <c r="I7" s="9">
+        <f t="shared" si="1"/>
         <v>2.3307083333333334</v>
       </c>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="10">
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="9">
         <f>Tableau1[[#This Row],[bénéfice]]*Tableau1[[#This Row],[% dons]]</f>
         <v>0.23307083333333334</v>
       </c>
-      <c r="O7" s="9">
+      <c r="O7" s="8">
         <v>0.1</v>
       </c>
-      <c r="P7" s="11">
+      <c r="P7" s="10">
         <f>Tableau1[[#This Row],[bénéfice]]-Tableau1[[#This Row],[dont asso]]</f>
         <v>2.0976375000000003</v>
       </c>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
-      <c r="S7" s="3"/>
-      <c r="T7" s="3"/>
-      <c r="U7" s="3"/>
-      <c r="V7" s="3"/>
-      <c r="W7" s="3"/>
-      <c r="X7" s="3"/>
-      <c r="Y7" s="3"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="2"/>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="2"/>
+      <c r="W7" s="2"/>
+      <c r="X7" s="2"/>
+      <c r="Y7" s="2"/>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="O8" s="3"/>
-      <c r="P8" s="3"/>
-      <c r="Q8" s="3"/>
-      <c r="R8" s="3"/>
-      <c r="S8" s="3"/>
-      <c r="T8" s="5"/>
-      <c r="U8" s="6"/>
-      <c r="V8" s="3"/>
-      <c r="W8" s="3"/>
-      <c r="X8" s="3"/>
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
+      <c r="S8" s="2"/>
+      <c r="T8" s="4"/>
+      <c r="U8" s="5"/>
+      <c r="V8" s="2"/>
+      <c r="W8" s="2"/>
+      <c r="X8" s="2"/>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="O9" s="3"/>
-      <c r="P9" s="3"/>
-      <c r="Q9" s="3"/>
-      <c r="R9" s="3"/>
-      <c r="S9" s="3"/>
-      <c r="T9" s="5"/>
-      <c r="U9" s="6"/>
-      <c r="V9" s="3"/>
-      <c r="W9" s="3"/>
-      <c r="X9" s="3"/>
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2"/>
+      <c r="S9" s="2"/>
+      <c r="T9" s="4"/>
+      <c r="U9" s="5"/>
+      <c r="V9" s="2"/>
+      <c r="W9" s="2"/>
+      <c r="X9" s="2"/>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-      <c r="O10" s="3"/>
-      <c r="P10" s="3"/>
-      <c r="Q10" s="3"/>
-      <c r="R10" s="3"/>
-      <c r="S10" s="3"/>
-      <c r="T10" s="3"/>
-      <c r="U10" s="3"/>
-      <c r="V10" s="3"/>
-      <c r="W10" s="3"/>
-      <c r="X10" s="3"/>
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
+      <c r="O10" s="2"/>
+      <c r="P10" s="2"/>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="2"/>
+      <c r="S10" s="2"/>
+      <c r="T10" s="2"/>
+      <c r="U10" s="2"/>
+      <c r="V10" s="2"/>
+      <c r="W10" s="2"/>
+      <c r="X10" s="2"/>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
-      <c r="O11" s="3"/>
-      <c r="P11" s="3"/>
-      <c r="Q11" s="3"/>
-      <c r="R11" s="3"/>
-      <c r="S11" s="3"/>
-      <c r="T11" s="3"/>
-      <c r="U11" s="3"/>
-      <c r="V11" s="3"/>
-      <c r="W11" s="3"/>
-      <c r="X11" s="3"/>
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2"/>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="R11" s="2"/>
+      <c r="S11" s="2"/>
+      <c r="T11" s="2"/>
+      <c r="U11" s="2"/>
+      <c r="V11" s="2"/>
+      <c r="W11" s="2"/>
+      <c r="X11" s="2"/>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-      <c r="M12" s="3"/>
-      <c r="N12" s="3"/>
-      <c r="O12" s="3"/>
-      <c r="P12" s="3"/>
-      <c r="Q12" s="3"/>
-      <c r="R12" s="3"/>
-      <c r="S12" s="3"/>
-      <c r="T12" s="3"/>
-      <c r="U12" s="3"/>
-      <c r="V12" s="3"/>
-      <c r="W12" s="3"/>
-      <c r="X12" s="3"/>
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
+      <c r="O12" s="2"/>
+      <c r="P12" s="2"/>
+      <c r="Q12" s="2"/>
+      <c r="R12" s="2"/>
+      <c r="S12" s="2"/>
+      <c r="T12" s="2"/>
+      <c r="U12" s="2"/>
+      <c r="V12" s="2"/>
+      <c r="W12" s="2"/>
+      <c r="X12" s="2"/>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-      <c r="O13" s="3"/>
-      <c r="P13" s="3"/>
-      <c r="Q13" s="3"/>
-      <c r="R13" s="3"/>
-      <c r="S13" s="3"/>
-      <c r="T13" s="3"/>
-      <c r="U13" s="3"/>
-      <c r="V13" s="3"/>
-      <c r="W13" s="3"/>
-      <c r="X13" s="3"/>
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2"/>
+      <c r="P13" s="2"/>
+      <c r="Q13" s="2"/>
+      <c r="R13" s="2"/>
+      <c r="S13" s="2"/>
+      <c r="T13" s="2"/>
+      <c r="U13" s="2"/>
+      <c r="V13" s="2"/>
+      <c r="W13" s="2"/>
+      <c r="X13" s="2"/>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
-      <c r="O14" s="3"/>
-      <c r="P14" s="3"/>
-      <c r="Q14" s="3"/>
-      <c r="R14" s="3"/>
-      <c r="S14" s="3"/>
-      <c r="T14" s="3"/>
-      <c r="U14" s="3"/>
-      <c r="V14" s="3"/>
-      <c r="W14" s="3"/>
-      <c r="X14" s="3"/>
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
+      <c r="N14" s="2"/>
+      <c r="O14" s="2"/>
+      <c r="P14" s="2"/>
+      <c r="Q14" s="2"/>
+      <c r="R14" s="2"/>
+      <c r="S14" s="2"/>
+      <c r="T14" s="2"/>
+      <c r="U14" s="2"/>
+      <c r="V14" s="2"/>
+      <c r="W14" s="2"/>
+      <c r="X14" s="2"/>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
-      <c r="O15" s="3"/>
-      <c r="P15" s="3"/>
-      <c r="Q15" s="3"/>
-      <c r="R15" s="3"/>
-      <c r="S15" s="3"/>
-      <c r="T15" s="3"/>
-      <c r="U15" s="3"/>
-      <c r="V15" s="3"/>
-      <c r="W15" s="3"/>
-      <c r="X15" s="3"/>
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
+      <c r="O15" s="2"/>
+      <c r="P15" s="2"/>
+      <c r="Q15" s="2"/>
+      <c r="R15" s="2"/>
+      <c r="S15" s="2"/>
+      <c r="T15" s="2"/>
+      <c r="U15" s="2"/>
+      <c r="V15" s="2"/>
+      <c r="W15" s="2"/>
+      <c r="X15" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1717,4 +2104,665 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AFE4FEB-1F95-4061-91E5-8B19782CFDAB}">
+  <dimension ref="A1:G31"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="7" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="32" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+    </row>
+    <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+    </row>
+    <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="31">
+        <v>0.21199999999999999</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" s="29">
+        <v>0.5</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B7" s="29">
+        <v>0.25</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="30">
+        <v>150</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="29">
+        <v>20</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+    </row>
+    <row r="12" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="G12" s="15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" s="27">
+        <v>15</v>
+      </c>
+      <c r="C13" s="28">
+        <v>0.5</v>
+      </c>
+      <c r="D13" s="24">
+        <f>B13*C13</f>
+        <v>7.5</v>
+      </c>
+      <c r="E13" s="27">
+        <v>15</v>
+      </c>
+      <c r="F13" s="24">
+        <f>E13*$B$5</f>
+        <v>3.1799999999999997</v>
+      </c>
+      <c r="G13" s="24">
+        <f>E13-D13-F13</f>
+        <v>4.32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="B14" s="27">
+        <v>20</v>
+      </c>
+      <c r="C14" s="28">
+        <v>1</v>
+      </c>
+      <c r="D14" s="24">
+        <f>B14*C14</f>
+        <v>20</v>
+      </c>
+      <c r="E14" s="27">
+        <v>30</v>
+      </c>
+      <c r="F14" s="24">
+        <f>E14*$B$5</f>
+        <v>6.3599999999999994</v>
+      </c>
+      <c r="G14" s="24">
+        <f>E14-D14-F14</f>
+        <v>3.6400000000000006</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" s="27">
+        <v>20</v>
+      </c>
+      <c r="C15" s="28">
+        <v>2</v>
+      </c>
+      <c r="D15" s="24">
+        <f>B15*C15</f>
+        <v>40</v>
+      </c>
+      <c r="E15" s="27">
+        <v>45</v>
+      </c>
+      <c r="F15" s="24">
+        <f>E15*$B$5</f>
+        <v>9.5399999999999991</v>
+      </c>
+      <c r="G15" s="24">
+        <f>E15-D15-F15</f>
+        <v>-4.5399999999999991</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" s="24">
+        <v>0</v>
+      </c>
+      <c r="C16" s="25">
+        <v>0</v>
+      </c>
+      <c r="D16" s="24">
+        <f>B16*C16</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="24">
+        <v>0</v>
+      </c>
+      <c r="F16" s="24">
+        <f>E16*$B$5</f>
+        <v>0</v>
+      </c>
+      <c r="G16" s="24">
+        <f>E16-D16-F16</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+    </row>
+    <row r="19" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="F19" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="G19" s="15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" s="23">
+        <v>150</v>
+      </c>
+      <c r="C20" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="19"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="12">
+        <f>(B20/1000)*$B$9</f>
+        <v>3</v>
+      </c>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="19"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="12">
+        <f>((HOUR(B21)+MINUTE(B21)/60)*($B$8/1000))*$B$7</f>
+        <v>0.24437499999999998</v>
+      </c>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
+      <c r="G23" s="19"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="12">
+        <f>(HOUR(B21)+MINUTE(B21)/60)*$B$6</f>
+        <v>3.2583333333333333</v>
+      </c>
+      <c r="E24" s="19"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="19"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="12">
+        <f>D22+D23+D24</f>
+        <v>6.5027083333333326</v>
+      </c>
+      <c r="E25" s="18">
+        <v>30</v>
+      </c>
+      <c r="F25" s="12">
+        <f>E25*$B$5</f>
+        <v>6.3599999999999994</v>
+      </c>
+      <c r="G25" s="12">
+        <f>E25-D25-F25</f>
+        <v>17.13729166666667</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="B28" s="16"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="16"/>
+    </row>
+    <row r="29" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" s="12">
+        <v>16.899999999999999</v>
+      </c>
+      <c r="C30" s="13">
+        <v>25</v>
+      </c>
+      <c r="D30" s="12">
+        <f>C30-B30</f>
+        <v>8.1000000000000014</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B31" s="12">
+        <v>22</v>
+      </c>
+      <c r="C31" s="13">
+        <v>32</v>
+      </c>
+      <c r="D31" s="12">
+        <f>C31-B31</f>
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="A28:G28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34B333BE-EABE-48E2-9697-BA4BA33D3938}">
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="42" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="6" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="32" t="s">
+        <v>106</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+    </row>
+    <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="46" t="s">
+        <v>105</v>
+      </c>
+      <c r="D3" s="46" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="45" t="s">
+        <v>103</v>
+      </c>
+      <c r="D4" s="45" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+    </row>
+    <row r="8" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="43" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="C9" s="44" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="41">
+        <v>1</v>
+      </c>
+      <c r="E9" s="24">
+        <f>VLOOKUP(C9, 'Calculs &amp; Barème'!$A$13:$E$15, 5, FALSE)</f>
+        <v>45</v>
+      </c>
+      <c r="F9" s="24">
+        <f>D9*E9</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="43" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10" s="42" t="s">
+        <v>86</v>
+      </c>
+      <c r="D10" s="41">
+        <v>1</v>
+      </c>
+      <c r="E10" s="24">
+        <v>0</v>
+      </c>
+      <c r="F10" s="24">
+        <f>D10*E10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="43" t="s">
+        <v>90</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C11" s="42" t="s">
+        <v>86</v>
+      </c>
+      <c r="D11" s="41">
+        <v>1</v>
+      </c>
+      <c r="E11" s="24">
+        <f>IF(C11="Oui", 'Calculs &amp; Barème'!E25, 0)</f>
+        <v>30</v>
+      </c>
+      <c r="F11" s="24">
+        <f>D11*E11</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="43" t="s">
+        <v>88</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="C12" s="42" t="s">
+        <v>86</v>
+      </c>
+      <c r="D12" s="41">
+        <v>1</v>
+      </c>
+      <c r="E12" s="24">
+        <f>IF(AND(C12="Oui", C11="Oui"), 'Calculs &amp; Barème'!C30, 0)</f>
+        <v>25</v>
+      </c>
+      <c r="F12" s="24">
+        <f>D12*E12</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E14" s="40" t="s">
+        <v>85</v>
+      </c>
+      <c r="F14" s="39">
+        <f>SUM(F9:F12)</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E15" s="38" t="s">
+        <v>84</v>
+      </c>
+      <c r="F15" s="37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="21" x14ac:dyDescent="0.25">
+      <c r="E16" s="36" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" s="35">
+        <f>F14+F15</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="B18" s="33"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="33"/>
+      <c r="B19" s="33"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="33"/>
+      <c r="B20" s="33"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="33"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="33"/>
+      <c r="B21" s="33"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="33"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="33"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A18:F21"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="list" sqref="C10:C12" xr:uid="{00000000-0002-0000-0100-000001000000}">
+      <formula1>"Oui,Non"</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="C9" xr:uid="{00000000-0002-0000-0100-000000000000}">
+      <formula1>"Conception simple,Reproduction technique,Conception technique"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>